<commit_message>
updated industry work flow
</commit_message>
<xml_diff>
--- a/industry/input_data/steel/Worldsteel-totalproductionofcrudesteel.xlsx
+++ b/industry/input_data/steel/Worldsteel-totalproductionofcrudesteel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fraunhofer-my.sharepoint.com/personal/rakesh_etikala_narendar_iee_fraunhofer_de/Documents/Desktop/sectoral-energy-demands/industry/input_data/steel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="11_3352B0E1F3F105F010E720AC36A94142DD0FB1ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D8E9E39-47C6-41DB-8ACC-69454DABC7A9}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="11_3352B0E1F3F105F010E720AC36A94142DD0FB1ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CBBB647C-AD30-4466-B410-8C18B8F655C2}"/>
   <bookViews>
-    <workbookView xWindow="1140" yWindow="1140" windowWidth="22320" windowHeight="17770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="20" yWindow="740" windowWidth="19180" windowHeight="11260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="P1_crude_steel_total_pub" sheetId="1" r:id="rId1"/>
@@ -1510,7 +1510,7 @@
         <v>492.64400000000001</v>
       </c>
     </row>
-    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>33</v>
       </c>
@@ -2350,7 +2350,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="77" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>75</v>
       </c>
@@ -2870,7 +2870,7 @@
         <v>594.61099999999999</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>101</v>
       </c>
@@ -3456,7 +3456,8 @@
   <autoFilter ref="A3:F128" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="0">
       <filters>
-        <filter val="South Africa"/>
+        <filter val="Egypt"/>
+        <filter val="Morocco"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>